<commit_message>
Call-center planner: add a baseline, README and review notes
- Baseline: the supervisor's fixed rota, drawn up without looking at the forecast.
- The under-staffing weight of 40 is explained as a business cost in every locale (number unchanged).
- The holiday is a regional public holiday in the main market; Korean wording fixed.
- The rejected leave request no longer shows a day above 12.
- README and REVIEW.md: the exact MILP optimum is normalized quality 1.18.

Open findings are proposals in the case's REVIEW.md.
</commit_message>
<xml_diff>
--- a/cases/customer_service/callcenter_workforce_planner/dataset/visible/ko/고객센터_상담원명단.xlsx
+++ b/cases/customer_service/callcenter_workforce_planner/dataset/visible/ko/고객센터_상담원명단.xlsx
@@ -452,7 +452,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -474,7 +474,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>정규직</t>
+          <t>풀타임</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">

</xml_diff>